<commit_message>
Add soldier 8129902 Yuvali Li
</commit_message>
<xml_diff>
--- a/src/data/alfon.xlsx
+++ b/src/data/alfon.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1615,9 +1615,35 @@
         <v>נגביסט</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>ב</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48" t="str">
+        <v>רובוטיקה</v>
+      </c>
+      <c r="D48" t="str">
+        <v>קצין</v>
+      </c>
+      <c r="E48">
+        <v>8129902</v>
+      </c>
+      <c r="F48" t="str">
+        <v>לי</v>
+      </c>
+      <c r="G48" t="str">
+        <v>יובלי</v>
+      </c>
+      <c r="H48" t="str">
+        <v>מפקד פלוגת רובוטיקה</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I48"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add soldier Itzhak Nissim Bitton (9124911) to roster
</commit_message>
<xml_diff>
--- a/src/data/alfon.xlsx
+++ b/src/data/alfon.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:K49"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,6 +427,12 @@
       <c r="I1" t="str">
         <v>__EMPTY</v>
       </c>
+      <c r="J1" t="str">
+        <v>שם מלא</v>
+      </c>
+      <c r="K1" t="str">
+        <v>מספר אישי</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1641,9 +1647,26 @@
         <v>מפקד פלוגת רובוטיקה</v>
       </c>
     </row>
+    <row r="49">
+      <c r="B49" t="str">
+        <v>מחלקה 1</v>
+      </c>
+      <c r="D49" t="str">
+        <v>סמר</v>
+      </c>
+      <c r="H49" t="str">
+        <v>מטול</v>
+      </c>
+      <c r="J49" t="str">
+        <v>יצחק ניסים ביטון</v>
+      </c>
+      <c r="K49" t="str">
+        <v>9124911</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K49"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>